<commit_message>
Updated MYS_grids_kan model - 2026-05-20 13:39
</commit_message>
<xml_diff>
--- a/VerveStacks_MYS_grids_kan/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_MYS_grids_kan/ReportDefs_vervestacks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\VEDA\Veda\Veda_models\vervestacks_models\VerveStacks_MYS_grids_kan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{09A7FC39-8B4B-4607-A447-CEE89292F52D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{5E8B1F13-42CB-4E70-86AF-3D9ECB54BBC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2730" yWindow="2730" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="geolocation" sheetId="72" r:id="rId1"/>
@@ -3949,7 +3949,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{67AE5CB7-D95C-4426-893C-4A8BF9F3D177}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B9322D8-9ED9-44D6-A8A7-499A9CD22A63}">
   <dimension ref="B9:H226"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
@@ -24420,7 +24420,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{18BA5BA9-71DC-44F8-AE2C-CE039B5DC984}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0D167F0E-5D67-42F0-A1B0-F1F1A0855AA5}">
   <dimension ref="B9:L226"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>

</xml_diff>